<commit_message>
📊 OLX Monitor 2026-03-02 09:34
</commit_message>
<xml_diff>
--- a/data/olx_monitoring.xlsx
+++ b/data/olx_monitoring.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -52,6 +52,10 @@
     <font>
       <b val="1"/>
       <color rgb="0047ffa0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00e8ff47"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -109,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -157,6 +161,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -525,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H269"/>
+  <dimension ref="A1:H278"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -10681,6 +10688,348 @@
         </is>
       </c>
       <c r="H269" t="inlineStr">
+        <is>
+          <t>mam-do-wynajecia-pokoj-dla-os-pracujacej-lub-studenta-narutowicza-14-CID3-ID18ySfv</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:34:30</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C270" s="13" t="inlineStr">
+        <is>
+          <t>Kawalerka po remoncie z funkcjonalną antresolą - ul. Jana Sawy</t>
+        </is>
+      </c>
+      <c r="D270" s="14" t="n">
+        <v>2499</v>
+      </c>
+      <c r="E270" s="14" t="inlineStr">
+        <is>
+          <t>28.10.2025</t>
+        </is>
+      </c>
+      <c r="F270" s="15" t="n">
+        <v>124</v>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/kawalerka-po-remoncie-z-funkcjonalna-antresola-ul-jana-sawy-CID3-ID183ger.html</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>kawalerka-po-remoncie-z-funkcjonalna-antresola-ul-jana-sawy-CID3-ID183ger</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:34:30</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C271" s="13" t="inlineStr">
+        <is>
+          <t>Duży pokój z balkonem w 2pokojowym mieszkaniu blisko Politechniki</t>
+        </is>
+      </c>
+      <c r="D271" s="14" t="n">
+        <v>1665</v>
+      </c>
+      <c r="E271" s="14" t="inlineStr">
+        <is>
+          <t>25.02.2026</t>
+        </is>
+      </c>
+      <c r="F271" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/duzy-pokoj-z-balkonem-w-2pokojowym-mieszkaniu-blisko-politechniki-CID3-ID19xpQK.html</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>duzy-pokoj-z-balkonem-w-2pokojowym-mieszkaniu-blisko-politechniki-CID3-ID19xpQK</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:34:30</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C272" s="13" t="inlineStr">
+        <is>
+          <t>Nowoczesne mieszkanie 2-pokojowe z balkonem, blisko UMCS, KUL, UP</t>
+        </is>
+      </c>
+      <c r="D272" s="14" t="n">
+        <v>2499</v>
+      </c>
+      <c r="E272" s="14" t="inlineStr">
+        <is>
+          <t>25.02.2026</t>
+        </is>
+      </c>
+      <c r="F272" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/nowoczesne-mieszkanie-2-pokojowe-z-balkonem-blisko-umcs-kul-up-CID3-ID19xpwN.html</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>nowoczesne-mieszkanie-2-pokojowe-z-balkonem-blisko-umcs-kul-up-CID3-ID19xpwN</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:34:30</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C273" s="13" t="inlineStr">
+        <is>
+          <t>Przytulny pokój blisko Politechniki – ul. Przytulna</t>
+        </is>
+      </c>
+      <c r="D273" s="14" t="n">
+        <v>549</v>
+      </c>
+      <c r="E273" s="14" t="inlineStr">
+        <is>
+          <t>10.10.2025</t>
+        </is>
+      </c>
+      <c r="F273" s="15" t="n">
+        <v>143</v>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/przytulny-pokoj-blisko-politechniki-ul-przytulna-CID3-ID17NeTz.html</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>przytulny-pokoj-blisko-politechniki-ul-przytulna-CID3-ID17NeTz</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:34:30</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C274" s="13" t="inlineStr">
+        <is>
+          <t>Mieszkanie z KLIMATYZACJĄ 5 minut od UMCS, UP, KUL - Długosza</t>
+        </is>
+      </c>
+      <c r="D274" s="14" t="n">
+        <v>2049</v>
+      </c>
+      <c r="E274" s="14" t="inlineStr">
+        <is>
+          <t>19.12.2025</t>
+        </is>
+      </c>
+      <c r="F274" s="15" t="n">
+        <v>72</v>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/mieszkanie-z-klimatyzacja-5-minut-od-umcs-up-kul-dlugosza-CID3-ID18KAEc.html</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>mieszkanie-z-klimatyzacja-5-minut-od-umcs-up-kul-dlugosza-CID3-ID18KAEc</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:34:30</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>pokojewlublinie</t>
+        </is>
+      </c>
+      <c r="C275" s="13" t="inlineStr">
+        <is>
+          <t>WOLNY OD ZARAZ! Super lokalizacja, blisko centrum, ul. Paganiniego 12</t>
+        </is>
+      </c>
+      <c r="D275" s="14" t="n">
+        <v>12640</v>
+      </c>
+      <c r="E275" s="14" t="inlineStr">
+        <is>
+          <t>19.01.2026</t>
+        </is>
+      </c>
+      <c r="F275" s="14" t="n">
+        <v>41</v>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/wolny-od-zaraz-super-lokalizacja-blisko-centrum-ul-paganiniego-12-CID3-ID195dLc.html</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>wolny-od-zaraz-super-lokalizacja-blisko-centrum-ul-paganiniego-12-CID3-ID195dLc</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:34:30</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>pokojewlublinie</t>
+        </is>
+      </c>
+      <c r="C276" s="13" t="inlineStr">
+        <is>
+          <t>WOLNY OD ZARAZ! Pokój jedynka, ul. Romanowskiego 58</t>
+        </is>
+      </c>
+      <c r="D276" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E276" s="14" t="inlineStr">
+        <is>
+          <t>11.08.2025</t>
+        </is>
+      </c>
+      <c r="F276" s="15" t="n">
+        <v>202</v>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/wolny-od-zaraz-pokoj-jedynka-ul-romanowskiego-58-CID3-ID16ZeYm.html</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>wolny-od-zaraz-pokoj-jedynka-ul-romanowskiego-58-CID3-ID16ZeYm</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:34:30</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>dawnypatron</t>
+        </is>
+      </c>
+      <c r="C277" s="13" t="inlineStr">
+        <is>
+          <t>Ładny pokój jednoosobowy. Wynajmę duży pokój w centrum. ul Niecała 4.</t>
+        </is>
+      </c>
+      <c r="D277" s="14" t="n">
+        <v>730</v>
+      </c>
+      <c r="E277" s="14" t="inlineStr">
+        <is>
+          <t>20.09.2024</t>
+        </is>
+      </c>
+      <c r="F277" s="15" t="n">
+        <v>527</v>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/ladny-pokoj-jednoosobowy-wynajme-duzy-pokoj-w-centrum-ul-niecala-4-CID3-ID122jPM.html</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>ladny-pokoj-jednoosobowy-wynajme-duzy-pokoj-w-centrum-ul-niecala-4-CID3-ID122jPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:34:30</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>dawnypatron</t>
+        </is>
+      </c>
+      <c r="C278" s="13" t="inlineStr">
+        <is>
+          <t>Mam do wynajęcia pokój dla os. pracującej lub studenta. Narutowicza 14</t>
+        </is>
+      </c>
+      <c r="D278" s="14" t="n">
+        <v>14690</v>
+      </c>
+      <c r="E278" s="14" t="inlineStr">
+        <is>
+          <t>05.12.2025</t>
+        </is>
+      </c>
+      <c r="F278" s="15" t="n">
+        <v>86</v>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/mam-do-wynajecia-pokoj-dla-os-pracujacej-lub-studenta-narutowicza-14-CID3-ID18ySfv.html</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
         <is>
           <t>mam-do-wynajecia-pokoj-dla-os-pracujacej-lub-studenta-narutowicza-14-CID3-ID18ySfv</t>
         </is>

</xml_diff>

<commit_message>
📊 OLX Monitor 2026-03-03 08:05
</commit_message>
<xml_diff>
--- a/data/olx_monitoring.xlsx
+++ b/data/olx_monitoring.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H278"/>
+  <dimension ref="A1:H287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11030,6 +11030,348 @@
         </is>
       </c>
       <c r="H278" t="inlineStr">
+        <is>
+          <t>mam-do-wynajecia-pokoj-dla-os-pracujacej-lub-studenta-narutowicza-14-CID3-ID18ySfv</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-03 08:05:48</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C279" s="13" t="inlineStr">
+        <is>
+          <t>Przytulny pokój blisko Politechniki – ul. Przytulna</t>
+        </is>
+      </c>
+      <c r="D279" s="14" t="n">
+        <v>549</v>
+      </c>
+      <c r="E279" s="14" t="inlineStr">
+        <is>
+          <t>10.10.2025</t>
+        </is>
+      </c>
+      <c r="F279" s="15" t="n">
+        <v>143</v>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/przytulny-pokoj-blisko-politechniki-ul-przytulna-CID3-ID17NeTz.html</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>przytulny-pokoj-blisko-politechniki-ul-przytulna-CID3-ID17NeTz</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-03 08:05:48</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C280" s="13" t="inlineStr">
+        <is>
+          <t>Duży pokój z balkonem w 2pokojowym mieszkaniu blisko Politechniki</t>
+        </is>
+      </c>
+      <c r="D280" s="14" t="n">
+        <v>1665</v>
+      </c>
+      <c r="E280" s="14" t="inlineStr">
+        <is>
+          <t>25.02.2026</t>
+        </is>
+      </c>
+      <c r="F280" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/duzy-pokoj-z-balkonem-w-2pokojowym-mieszkaniu-blisko-politechniki-CID3-ID19xpQK.html</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>duzy-pokoj-z-balkonem-w-2pokojowym-mieszkaniu-blisko-politechniki-CID3-ID19xpQK</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-03 08:05:48</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C281" s="13" t="inlineStr">
+        <is>
+          <t>Mieszkanie z KLIMATYZACJĄ 5 minut od UMCS, UP, KUL - Długosza</t>
+        </is>
+      </c>
+      <c r="D281" s="14" t="n">
+        <v>2049</v>
+      </c>
+      <c r="E281" s="14" t="inlineStr">
+        <is>
+          <t>19.12.2025</t>
+        </is>
+      </c>
+      <c r="F281" s="15" t="n">
+        <v>73</v>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/mieszkanie-z-klimatyzacja-5-minut-od-umcs-up-kul-dlugosza-CID3-ID18KAEc.html</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>mieszkanie-z-klimatyzacja-5-minut-od-umcs-up-kul-dlugosza-CID3-ID18KAEc</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-03 08:05:48</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C282" s="13" t="inlineStr">
+        <is>
+          <t>Nowoczesne mieszkanie 2-pokojowe z balkonem, blisko UMCS, KUL, UP</t>
+        </is>
+      </c>
+      <c r="D282" s="14" t="n">
+        <v>2499</v>
+      </c>
+      <c r="E282" s="14" t="inlineStr">
+        <is>
+          <t>25.02.2026</t>
+        </is>
+      </c>
+      <c r="F282" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/nowoczesne-mieszkanie-2-pokojowe-z-balkonem-blisko-umcs-kul-up-CID3-ID19xpwN.html</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>nowoczesne-mieszkanie-2-pokojowe-z-balkonem-blisko-umcs-kul-up-CID3-ID19xpwN</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-03 08:05:48</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C283" s="13" t="inlineStr">
+        <is>
+          <t>Kawalerka po remoncie z funkcjonalną antresolą - ul. Jana Sawy</t>
+        </is>
+      </c>
+      <c r="D283" s="14" t="n">
+        <v>2499</v>
+      </c>
+      <c r="E283" s="14" t="inlineStr">
+        <is>
+          <t>28.10.2025</t>
+        </is>
+      </c>
+      <c r="F283" s="15" t="n">
+        <v>125</v>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/kawalerka-po-remoncie-z-funkcjonalna-antresola-ul-jana-sawy-CID3-ID183ger.html</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>kawalerka-po-remoncie-z-funkcjonalna-antresola-ul-jana-sawy-CID3-ID183ger</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-03 08:05:48</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>pokojewlublinie</t>
+        </is>
+      </c>
+      <c r="C284" s="13" t="inlineStr">
+        <is>
+          <t>WOLNY OD ZARAZ! Pokój jedynka, ul. Romanowskiego 58</t>
+        </is>
+      </c>
+      <c r="D284" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E284" s="14" t="inlineStr">
+        <is>
+          <t>11.08.2025</t>
+        </is>
+      </c>
+      <c r="F284" s="15" t="n">
+        <v>203</v>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/wolny-od-zaraz-pokoj-jedynka-ul-romanowskiego-58-CID3-ID16ZeYm.html</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>wolny-od-zaraz-pokoj-jedynka-ul-romanowskiego-58-CID3-ID16ZeYm</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-03 08:05:48</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>pokojewlublinie</t>
+        </is>
+      </c>
+      <c r="C285" s="13" t="inlineStr">
+        <is>
+          <t>WOLNY OD ZARAZ! Super lokalizacja, blisko centrum, ul. Paganiniego 12</t>
+        </is>
+      </c>
+      <c r="D285" s="14" t="n">
+        <v>12640</v>
+      </c>
+      <c r="E285" s="14" t="inlineStr">
+        <is>
+          <t>19.01.2026</t>
+        </is>
+      </c>
+      <c r="F285" s="14" t="n">
+        <v>42</v>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/wolny-od-zaraz-super-lokalizacja-blisko-centrum-ul-paganiniego-12-CID3-ID195dLc.html</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>wolny-od-zaraz-super-lokalizacja-blisko-centrum-ul-paganiniego-12-CID3-ID195dLc</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-03 08:05:48</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>dawnypatron</t>
+        </is>
+      </c>
+      <c r="C286" s="13" t="inlineStr">
+        <is>
+          <t>Ładny pokój jednoosobowy. Wynajmę duży pokój w centrum. ul Niecała 4.</t>
+        </is>
+      </c>
+      <c r="D286" s="14" t="n">
+        <v>730</v>
+      </c>
+      <c r="E286" s="14" t="inlineStr">
+        <is>
+          <t>20.09.2024</t>
+        </is>
+      </c>
+      <c r="F286" s="15" t="n">
+        <v>528</v>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/ladny-pokoj-jednoosobowy-wynajme-duzy-pokoj-w-centrum-ul-niecala-4-CID3-ID122jPM.html</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>ladny-pokoj-jednoosobowy-wynajme-duzy-pokoj-w-centrum-ul-niecala-4-CID3-ID122jPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-03 08:05:48</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>dawnypatron</t>
+        </is>
+      </c>
+      <c r="C287" s="13" t="inlineStr">
+        <is>
+          <t>Mam do wynajęcia pokój dla os. pracującej lub studenta. Narutowicza 14</t>
+        </is>
+      </c>
+      <c r="D287" s="14" t="n">
+        <v>14690</v>
+      </c>
+      <c r="E287" s="14" t="inlineStr">
+        <is>
+          <t>05.12.2025</t>
+        </is>
+      </c>
+      <c r="F287" s="15" t="n">
+        <v>87</v>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/mam-do-wynajecia-pokoj-dla-os-pracujacej-lub-studenta-narutowicza-14-CID3-ID18ySfv.html</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
         <is>
           <t>mam-do-wynajecia-pokoj-dla-os-pracujacej-lub-studenta-narutowicza-14-CID3-ID18ySfv</t>
         </is>

</xml_diff>

<commit_message>
📊 OLX Monitor 2026-03-04 08:03
</commit_message>
<xml_diff>
--- a/data/olx_monitoring.xlsx
+++ b/data/olx_monitoring.xlsx
@@ -532,7 +532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H287"/>
+  <dimension ref="A1:H297"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11372,6 +11372,386 @@
         </is>
       </c>
       <c r="H287" t="inlineStr">
+        <is>
+          <t>mam-do-wynajecia-pokoj-dla-os-pracujacej-lub-studenta-narutowicza-14-CID3-ID18ySfv</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>artymiuk</t>
+        </is>
+      </c>
+      <c r="C288" s="13" t="inlineStr">
+        <is>
+          <t>Pokój z balkonem i widokiem na Ratusz – Ścisłe Centrum</t>
+        </is>
+      </c>
+      <c r="D288" s="14" t="n">
+        <v>1300</v>
+      </c>
+      <c r="E288" s="14" t="inlineStr">
+        <is>
+          <t>03.03.2026</t>
+        </is>
+      </c>
+      <c r="F288" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/pokoj-z-balkonem-i-widokiem-na-ratusz-scisle-centrum-CID3-ID19ClP1.html</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>pokoj-z-balkonem-i-widokiem-na-ratusz-scisle-centrum-CID3-ID19ClP1</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C289" s="13" t="inlineStr">
+        <is>
+          <t>Przytulny pokój blisko Politechniki – ul. Przytulna</t>
+        </is>
+      </c>
+      <c r="D289" s="14" t="n">
+        <v>549</v>
+      </c>
+      <c r="E289" s="14" t="inlineStr">
+        <is>
+          <t>10.10.2025</t>
+        </is>
+      </c>
+      <c r="F289" s="15" t="n">
+        <v>144</v>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/przytulny-pokoj-blisko-politechniki-ul-przytulna-CID3-ID17NeTz.html</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>przytulny-pokoj-blisko-politechniki-ul-przytulna-CID3-ID17NeTz</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C290" s="13" t="inlineStr">
+        <is>
+          <t>Duży pokój z balkonem w 2pokojowym mieszkaniu blisko Politechniki</t>
+        </is>
+      </c>
+      <c r="D290" s="14" t="n">
+        <v>1665</v>
+      </c>
+      <c r="E290" s="14" t="inlineStr">
+        <is>
+          <t>25.02.2026</t>
+        </is>
+      </c>
+      <c r="F290" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/duzy-pokoj-z-balkonem-w-2pokojowym-mieszkaniu-blisko-politechniki-CID3-ID19xpQK.html</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>duzy-pokoj-z-balkonem-w-2pokojowym-mieszkaniu-blisko-politechniki-CID3-ID19xpQK</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C291" s="13" t="inlineStr">
+        <is>
+          <t>Mieszkanie z KLIMATYZACJĄ 5 minut od UMCS, UP, KUL - Długosza</t>
+        </is>
+      </c>
+      <c r="D291" s="14" t="n">
+        <v>2049</v>
+      </c>
+      <c r="E291" s="14" t="inlineStr">
+        <is>
+          <t>19.12.2025</t>
+        </is>
+      </c>
+      <c r="F291" s="15" t="n">
+        <v>74</v>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/mieszkanie-z-klimatyzacja-5-minut-od-umcs-up-kul-dlugosza-CID3-ID18KAEc.html</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>mieszkanie-z-klimatyzacja-5-minut-od-umcs-up-kul-dlugosza-CID3-ID18KAEc</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C292" s="13" t="inlineStr">
+        <is>
+          <t>Nowoczesne mieszkanie 2-pokojowe z balkonem, blisko UMCS, KUL, UP</t>
+        </is>
+      </c>
+      <c r="D292" s="14" t="n">
+        <v>2499</v>
+      </c>
+      <c r="E292" s="14" t="inlineStr">
+        <is>
+          <t>25.02.2026</t>
+        </is>
+      </c>
+      <c r="F292" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/nowoczesne-mieszkanie-2-pokojowe-z-balkonem-blisko-umcs-kul-up-CID3-ID19xpwN.html</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>nowoczesne-mieszkanie-2-pokojowe-z-balkonem-blisko-umcs-kul-up-CID3-ID19xpwN</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>poqui</t>
+        </is>
+      </c>
+      <c r="C293" s="13" t="inlineStr">
+        <is>
+          <t>Kawalerka po remoncie z funkcjonalną antresolą - ul. Jana Sawy</t>
+        </is>
+      </c>
+      <c r="D293" s="14" t="n">
+        <v>2499</v>
+      </c>
+      <c r="E293" s="14" t="inlineStr">
+        <is>
+          <t>28.10.2025</t>
+        </is>
+      </c>
+      <c r="F293" s="15" t="n">
+        <v>126</v>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/kawalerka-po-remoncie-z-funkcjonalna-antresola-ul-jana-sawy-CID3-ID183ger.html</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>kawalerka-po-remoncie-z-funkcjonalna-antresola-ul-jana-sawy-CID3-ID183ger</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>pokojewlublinie</t>
+        </is>
+      </c>
+      <c r="C294" s="13" t="inlineStr">
+        <is>
+          <t>WOLNY OD ZARAZ! Super lokalizacja, blisko centrum, ul. Paganiniego 12</t>
+        </is>
+      </c>
+      <c r="D294" s="14" t="n">
+        <v>12640</v>
+      </c>
+      <c r="E294" s="14" t="inlineStr">
+        <is>
+          <t>19.01.2026</t>
+        </is>
+      </c>
+      <c r="F294" s="14" t="n">
+        <v>43</v>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/wolny-od-zaraz-super-lokalizacja-blisko-centrum-ul-paganiniego-12-CID3-ID195dLc.html</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>wolny-od-zaraz-super-lokalizacja-blisko-centrum-ul-paganiniego-12-CID3-ID195dLc</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>pokojewlublinie</t>
+        </is>
+      </c>
+      <c r="C295" s="13" t="inlineStr">
+        <is>
+          <t>WOLNY OD ZARAZ! Pokój jedynka, ul. Romanowskiego 58</t>
+        </is>
+      </c>
+      <c r="D295" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E295" s="14" t="inlineStr">
+        <is>
+          <t>11.08.2025</t>
+        </is>
+      </c>
+      <c r="F295" s="15" t="n">
+        <v>204</v>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/wolny-od-zaraz-pokoj-jedynka-ul-romanowskiego-58-CID3-ID16ZeYm.html</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>wolny-od-zaraz-pokoj-jedynka-ul-romanowskiego-58-CID3-ID16ZeYm</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>dawnypatron</t>
+        </is>
+      </c>
+      <c r="C296" s="13" t="inlineStr">
+        <is>
+          <t>Ładny pokój jednoosobowy. Wynajmę duży pokój w centrum. ul Niecała 4.</t>
+        </is>
+      </c>
+      <c r="D296" s="14" t="n">
+        <v>730</v>
+      </c>
+      <c r="E296" s="14" t="inlineStr">
+        <is>
+          <t>20.09.2024</t>
+        </is>
+      </c>
+      <c r="F296" s="15" t="n">
+        <v>529</v>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/ladny-pokoj-jednoosobowy-wynajme-duzy-pokoj-w-centrum-ul-niecala-4-CID3-ID122jPM.html</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>ladny-pokoj-jednoosobowy-wynajme-duzy-pokoj-w-centrum-ul-niecala-4-CID3-ID122jPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="13" t="inlineStr">
+        <is>
+          <t>2026-03-04 08:03:10</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>dawnypatron</t>
+        </is>
+      </c>
+      <c r="C297" s="13" t="inlineStr">
+        <is>
+          <t>Mam do wynajęcia pokój dla os. pracującej lub studenta. Narutowicza 14</t>
+        </is>
+      </c>
+      <c r="D297" s="14" t="n">
+        <v>14690</v>
+      </c>
+      <c r="E297" s="14" t="inlineStr">
+        <is>
+          <t>05.12.2025</t>
+        </is>
+      </c>
+      <c r="F297" s="15" t="n">
+        <v>88</v>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>https://www.olx.pl/d/oferta/mam-do-wynajecia-pokoj-dla-os-pracujacej-lub-studenta-narutowicza-14-CID3-ID18ySfv.html</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
         <is>
           <t>mam-do-wynajecia-pokoj-dla-os-pracujacej-lub-studenta-narutowicza-14-CID3-ID18ySfv</t>
         </is>

</xml_diff>